<commit_message>
Add email delivery helper for DeafLink scraper results
- Implemented `mailer.py` to handle email sending with job search results.
- Integrated environment variable loading for email credentials.
- Created HTML templates for email content, including summary and job listings.
- Added functions for generating summary tables and job previews from scraped data.
- Included error handling for missing credentials and attachment checks.
</commit_message>
<xml_diff>
--- a/output/atypical.xlsx
+++ b/output/atypical.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -543,12 +543,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HR Intern</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aditya Birla Chemicals</t>
+          <t>Global &amp; Corporate Banking</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>internship</t>
+          <t>job</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -579,24 +579,16 @@
           <t>custom_api</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15,000/-PM</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>15000</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/hr-intern-aditya-birla-chemicals-mumbai-1028</t>
+          <t>https://atypicaladvantage.in/find-a-job/sales-manager-global-corporate-banking-mumbai-1031</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -606,24 +598,24 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Jobs only for Person with Disability (PwD) Role: HR Intern Basic responsibilities: * Help with basic recruitment activities such as sourcing from job portals, interview coordination and candidate follow‑ups and update trackers * Support employer branding by coordinating collection of employee storie</t>
+          <t>Job Title: Sales Manager Location: Mumbai Role Description A Sales manager (Assets &amp; Liability Products) manages telephonic campaigns to acquire new customers and retain existing ones. The role focuses on selling retail loan products (Assets) and mobilizing low-cost deposits (Liabilities) to meet as</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Sr Analyst - Data Science</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Marico</t>
+          <t>Cardinal Health</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pan India</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="D3" t="b">
@@ -658,7 +650,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/trainee-marico-pan-india-1027</t>
+          <t>https://atypicaladvantage.in/find-a-job/sr-analyst-data-science-cardinal-health-bangalore-1029</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -668,24 +660,24 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Jobs for PwD About the Program: The WINGS Trainee Hiring Program is a 12-month structured traineeship designed to develop high-potential engineering graduates into future leaders. The program offers hands-on experience through long-term projects, providing exposure across corporate functions and man</t>
+          <t>Job Overview: Responsibilities As Data / Machine learning analyst work hands-on and together with external and internal partners to develop, test and operationalize data science and analytical solutions as well as ensure its adoption by businesses. Work to leverage data (Transactional / Big Data, Ex</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PLCS – Growth</t>
+          <t>HR Intern</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Leading Financial Services Organization</t>
+          <t>Aditya Birla Chemicals</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -693,7 +685,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>internship</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -711,16 +703,24 @@
           <t>custom_api</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15,000/-PM</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>15000</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/plcs-growth-leading-financial-services-organization-pune-1026</t>
+          <t>https://atypicaladvantage.in/find-a-job/hr-intern-aditya-birla-chemicals-mumbai-1028</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -730,24 +730,24 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Key Responsibilities: - Analyze large datasets to derive meaningful insights and support business growth - Develop and maintain reports, dashboards, and MIS using Advanced Excel and other tools - Write and optimize SQL queries for data extraction and analysis - Work with Python for data processing,</t>
+          <t>Jobs only for Person with Disability (PwD) Role: HR Intern Basic responsibilities: * Help with basic recruitment activities such as sourcing from job portals, interview coordination and candidate follow‑ups and update trackers * Support employer branding by coordinating collection of employee storie</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Senior Analyst, Facility and Security Technology</t>
+          <t>Trainee</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cardinal Health</t>
+          <t>Marico</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Pan India</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -782,7 +782,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/senior-analyst-facility-and-security-technology-cardinal-health-bangalore-1025</t>
+          <t>https://atypicaladvantage.in/find-a-job/trainee-marico-pan-india-1027</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -792,24 +792,24 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>What Facility and Security Technology contribute: Security implements measures to safeguard the company's assets from circumstances and threats that would cause harm or loss. Facility and Security Technology provides technical solutions for facility and security risk management. Creates security sta</t>
+          <t>Jobs for PwD About the Program: The WINGS Trainee Hiring Program is a 12-month structured traineeship designed to develop high-potential engineering graduates into future leaders. The program offers hands-on experience through long-term projects, providing exposure across corporate functions and man</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Engineer, IT Quality Control</t>
+          <t>PLCS – Growth</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cardinal Health</t>
+          <t>Leading Financial Services Organization</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -844,7 +844,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/engineer-it-quality-control-cardinal-health-bangalore-1023</t>
+          <t>https://atypicaladvantage.in/find-a-job/plcs-growth-leading-financial-services-organization-pune-1026</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -854,14 +854,14 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Qualifications: • BA, BS or equivalent experience in related field. Advance Degree preferred • Bachelor’s degree in Electronics, Computer Science, Computer Engineering or a software-related discipline. • 5+ years as a software automation tester. What is expected of you and others at this level • App</t>
+          <t>Key Responsibilities: - Analyze large datasets to derive meaningful insights and support business growth - Develop and maintain reports, dashboards, and MIS using Advanced Excel and other tools - Write and optimize SQL queries for data extraction and analysis - Work with Python for data processing,</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Senior Analyst, Facility and Security Technology</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -906,7 +906,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/full-stack-developer-cardinal-health-bangalore-1021</t>
+          <t>https://atypicaladvantage.in/find-a-job/senior-analyst-facility-and-security-technology-cardinal-health-bangalore-1025</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -916,24 +916,24 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Software Engineering is responsible for designing, developing, implementing and supporting applications, systems and IT products required to achieve the company's business objectives. Objectives:  Demonstrates knowledge of software development techniques and fluency in software languages and applic</t>
+          <t>What Facility and Security Technology contribute: Security implements measures to safeguard the company's assets from circumstances and threats that would cause harm or loss. Facility and Security Technology provides technical solutions for facility and security risk management. Creates security sta</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Copy Intern</t>
+          <t>Engineer, IT Quality Control</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Havas</t>
+          <t>Cardinal Health</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bangalore, Mumbai, Gurugram</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -941,7 +941,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>internship</t>
+          <t>job</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -959,24 +959,16 @@
           <t>custom_api</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>₹15,000 per month</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K8" t="n">
-        <v>15000</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/copy-intern-havas-bangalore-mumbai-gurugram-1020</t>
+          <t>https://atypicaladvantage.in/find-a-job/engineer-it-quality-control-cardinal-health-bangalore-1023</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -986,24 +978,24 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Job only for Person with Disability (PwD) Title: Copy Intern Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate - Exper</t>
+          <t>Qualifications: • BA, BS or equivalent experience in related field. Advance Degree preferred • Bachelor’s degree in Electronics, Computer Science, Computer Engineering or a software-related discipline. • 5+ years as a software automation tester. What is expected of you and others at this level • App</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Graphic Designer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Havas</t>
+          <t>Cardinal Health</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bangalore, Mumbai</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -1029,24 +1021,16 @@
           <t>custom_api</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>₹15,000 per month</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="n">
-        <v>180000</v>
-      </c>
-      <c r="M9" t="n">
-        <v>180000</v>
-      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/graphic-designer-havas-bangalore-mumbai-1019</t>
+          <t>https://atypicaladvantage.in/find-a-job/full-stack-developer-cardinal-health-bangalore-1021</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1056,14 +1040,14 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Job only for Person with Disability (PwD) Job Title: Graphic Designer Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduat</t>
+          <t>Software Engineering is responsible for designing, developing, implementing and supporting applications, systems and IT products required to achieve the company's business objectives. Objectives:  Demonstrates knowledge of software development techniques and fluency in software languages and applic</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Media Analyst</t>
+          <t>Copy Intern</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1073,7 +1057,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Bangalore, Mumbai, Gurugram</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -1081,7 +1065,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>internship</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1104,19 +1088,19 @@
           <t>₹15,000 per month</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="n">
-        <v>180000</v>
-      </c>
-      <c r="M10" t="n">
-        <v>180000</v>
-      </c>
+      <c r="J10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/media-analyst-havas-mumbai-1018</t>
+          <t>https://atypicaladvantage.in/find-a-job/copy-intern-havas-bangalore-mumbai-gurugram-1020</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1126,14 +1110,14 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Job only for Person with Disability (PwD) Job Title: Media Analyst Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate -</t>
+          <t>Job only for Person with Disability (PwD) Title: Copy Intern Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate - Exper</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Social Media Intern</t>
+          <t>Graphic Designer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1143,7 +1127,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Bangalore, Mumbai</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -1151,7 +1135,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>internship</t>
+          <t>job</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1174,19 +1158,19 @@
           <t>₹15,000 per month</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K11" t="n">
-        <v>15000</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>180000</v>
+      </c>
+      <c r="M11" t="n">
+        <v>180000</v>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/social-media-intern-havas-mumbai-1016</t>
+          <t>https://atypicaladvantage.in/find-a-job/graphic-designer-havas-bangalore-mumbai-1019</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1196,14 +1180,14 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Job only for Person with Disability (PwD) Job Title: Social Media Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate -</t>
+          <t>Job only for Person with Disability (PwD) Job Title: Graphic Designer Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduat</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PPT Designer</t>
+          <t>Media Analyst</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1256,7 +1240,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/ppt-designer-havas-mumbai-1015</t>
+          <t>https://atypicaladvantage.in/find-a-job/media-analyst-havas-mumbai-1018</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1266,19 +1250,19 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Job only for Person with Disability (PwD) Title: PPT Designer Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate - Expe</t>
+          <t>Job only for Person with Disability (PwD) Job Title: Media Analyst Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate -</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Human Resources Intern</t>
+          <t>Social Media Intern</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aditya Birla Chemicals</t>
+          <t>Havas</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1311,14 +1295,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>: 15-16k/PM</t>
+          <t>₹15,000 per month</t>
         </is>
       </c>
       <c r="J13" t="n">
         <v>15000</v>
       </c>
       <c r="K13" t="n">
-        <v>16000</v>
+        <v>15000</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1326,7 +1310,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>https://atypicaladvantage.in/find-a-job/human-resources-intern-aditya-birla-chemicals-mumbai-1012</t>
+          <t>https://atypicaladvantage.in/find-a-job/social-media-intern-havas-mumbai-1016</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1336,24 +1320,24 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Role : HR Intern Duration : 6 months Qualification : Any graduation Experience : Preferred, freshers and those with up to 2 years of experience can apply Location : Prabhadevi, Mumbai Basic responsibilities: - Help with basic recruitment activities such as sourcing from job portals, interview coordi</t>
+          <t>Job only for Person with Disability (PwD) Job Title: Social Media Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate -</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WILP - Work Integrated Learning Program</t>
+          <t>PPT Designer</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Havas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pan India</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -1381,26 +1365,166 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>No stipend during pre-skilling</t>
+          <t>₹15,000 per month</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>180000</v>
+      </c>
+      <c r="M14" t="n">
+        <v>180000</v>
+      </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
+          <t>https://atypicaladvantage.in/find-a-job/ppt-designer-havas-mumbai-1015</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>atypical</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Job only for Person with Disability (PwD) Title: PPT Designer Company: Havas Location: Gurugram | Mumbai | Bangalore Stipend: ₹15,000 per month Duration: 3 Months Type - Internship with FTE performance basis Work Mode: Work From Office (9:30 AM – 6:00 PM) Eligibility - Education: Any Graduate - Expe</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Human Resources Intern</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Aditya Birla Chemicals</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>explicit_pwd</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>custom_api</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>: 15-16k/PM</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K15" t="n">
+        <v>16000</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>https://atypicaladvantage.in/find-a-job/human-resources-intern-aditya-birla-chemicals-mumbai-1012</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>atypical</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Role : HR Intern Duration : 6 months Qualification : Any graduation Experience : Preferred, freshers and those with up to 2 years of experience can apply Location : Prabhadevi, Mumbai Basic responsibilities: - Help with basic recruitment activities such as sourcing from job portals, interview coordi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WILP - Work Integrated Learning Program</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pan India</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>job</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>explicit_pwd</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>custom_api</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No stipend during pre-skilling</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
           <t>https://atypicaladvantage.in/find-a-job/wilp-work-integrated-learning-program-wipro-pan-india-1004</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>atypical</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>Role Title: WILP Function: Technology Employment Type: Full-time (post successful completion of selection &amp; pre-skilling) Hiring Scope: PAN India Role Purpose We are looking to hire BCA/BSc graduates who are eager to start their professional technology careers through a structured early-career progr</t>
         </is>

</xml_diff>